<commit_message>
fix(checklist): corrigir mapeamento por ancoras, colunas de evidencias H, titulos e modalidade
</commit_message>
<xml_diff>
--- a/Checklist_Auditoria_ISO_13485_2016_3 (1).xlsx
+++ b/Checklist_Auditoria_ISO_13485_2016_3 (1).xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="20115" windowHeight="6045" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Check-List" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidências" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resultados" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="atenção" sheetId="4" state="hidden" r:id="rId4"/>
+    <sheet name="Check-List" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Evidências" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Resultados" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="atenção" sheetId="4" state="hidden" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="bd">#REF!</definedName>
@@ -26,7 +26,7 @@
     <numFmt numFmtId="164" formatCode="d\.m"/>
     <numFmt numFmtId="165" formatCode="0.0"/>
   </numFmts>
-  <fonts count="43">
+  <fonts count="44">
     <font>
       <name val="Arial"/>
       <color rgb="FF000000"/>
@@ -263,8 +263,14 @@
       <color rgb="0064748B"/>
       <sz val="9.5"/>
     </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="00000000"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="12">
+  <fills count="13">
     <fill>
       <patternFill/>
     </fill>
@@ -331,8 +337,14 @@
         <bgColor rgb="00F8FAFC"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9D9D9"/>
+        <bgColor rgb="00D9D9D9"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="19">
+  <borders count="23">
     <border>
       <left/>
       <right/>
@@ -545,11 +557,55 @@
         <color rgb="00CBD5E1"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00CBD5E1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00CBD5E1"/>
+      </right>
+      <top style="thin">
+        <color rgb="00CBD5E1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00CBD5E1"/>
+      </right>
+      <top style="thin">
+        <color rgb="00CBD5E1"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00CBD5E1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00CBD5E1"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00CBD5E1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="178">
+  <cellXfs count="186">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -1032,6 +1088,20 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="16" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="43" fillId="0" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="43" fillId="12" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="43" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="43" fillId="12" borderId="22" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="43" fillId="12" borderId="21" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1109,7 +1179,7 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <plotArea>
       <layout>
@@ -1145,7 +1215,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" cmpd="sng">
+            <a:ln cmpd="sng">
               <a:solidFill>
                 <a:srgbClr val="4285F4"/>
               </a:solidFill>
@@ -1155,7 +1225,7 @@
           <marker>
             <symbol val="none"/>
             <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:ln>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
@@ -1226,7 +1296,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" cmpd="sng">
+            <a:ln cmpd="sng">
               <a:solidFill>
                 <a:srgbClr val="EA4335"/>
               </a:solidFill>
@@ -1236,7 +1306,7 @@
           <marker>
             <symbol val="none"/>
             <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:ln>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
@@ -1307,7 +1377,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" cmpd="sng">
+            <a:ln cmpd="sng">
               <a:solidFill>
                 <a:srgbClr val="FBBC04"/>
               </a:solidFill>
@@ -1318,10 +1388,10 @@
             <symbol val="circle"/>
             <size val="10"/>
             <spPr>
-              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:solidFill>
                 <a:srgbClr val="FBBC04"/>
               </a:solidFill>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" cmpd="sng">
+              <a:ln cmpd="sng">
                 <a:solidFill>
                   <a:srgbClr val="FBBC04"/>
                 </a:solidFill>
@@ -1398,9 +1468,9 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr/>
+              <a:lstStyle/>
+              <a:p>
                 <a:pPr lvl="0">
                   <a:defRPr b="0">
                     <a:solidFill>
@@ -1410,7 +1480,7 @@
                   </a:defRPr>
                 </a:pPr>
                 <a:r>
-                  <a:t/>
+                  <a:t>None</a:t>
                 </a:r>
                 <a:endParaRPr lang="pt-BR"/>
               </a:p>
@@ -1424,9 +1494,9 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <txPr>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr lvl="0">
               <a:defRPr b="0">
                 <a:solidFill>
@@ -1436,7 +1506,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t/>
+              <a:t>None</a:t>
             </a:r>
             <a:endParaRPr lang="pt-BR"/>
           </a:p>
@@ -1457,7 +1527,7 @@
         <axPos val="l"/>
         <majorGridlines>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ln>
               <a:solidFill>
                 <a:srgbClr val="B7B7B7"/>
               </a:solidFill>
@@ -1467,7 +1537,7 @@
         </majorGridlines>
         <minorGridlines>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ln>
               <a:solidFill>
                 <a:srgbClr val="CCCCCC"/>
               </a:solidFill>
@@ -1478,9 +1548,9 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr/>
+              <a:lstStyle/>
+              <a:p>
                 <a:pPr lvl="0">
                   <a:defRPr b="0">
                     <a:solidFill>
@@ -1490,7 +1560,7 @@
                   </a:defRPr>
                 </a:pPr>
                 <a:r>
-                  <a:t/>
+                  <a:t>None</a:t>
                 </a:r>
                 <a:endParaRPr lang="pt-BR"/>
               </a:p>
@@ -1504,14 +1574,14 @@
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
         <spPr>
-          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:ln>
             <a:prstDash val="solid"/>
           </a:ln>
         </spPr>
         <txPr>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
             <a:pPr lvl="0">
               <a:defRPr b="0">
                 <a:solidFill>
@@ -1521,7 +1591,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t/>
+              <a:t>None</a:t>
             </a:r>
             <a:endParaRPr lang="pt-BR"/>
           </a:p>
@@ -1536,9 +1606,9 @@
       <layout/>
       <overlay val="0"/>
       <txPr>
-        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:bodyPr/>
+        <a:lstStyle/>
+        <a:p>
           <a:pPr lvl="0">
             <a:defRPr sz="1000" b="0">
               <a:solidFill>
@@ -1548,7 +1618,7 @@
             </a:defRPr>
           </a:pPr>
           <a:r>
-            <a:t/>
+            <a:t>None</a:t>
           </a:r>
           <a:endParaRPr lang="pt-BR"/>
         </a:p>
@@ -1561,47 +1631,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
-  <oneCellAnchor>
-    <from>
-      <col>1</col>
-      <colOff>47625</colOff>
-      <row>1</row>
-      <rowOff>228600</rowOff>
-    </from>
-    <ext cx="1819275" cy="190500"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="2" name="image1.png"/>
-        <cNvPicPr preferRelativeResize="0"/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:off x="123825" y="285750"/>
-          <a:ext cx="1819275" cy="190500"/>
-        </a:xfrm>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
-          <avLst/>
-        </a:prstGeom>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </spPr>
-    </pic>
-    <clientData fLocksWithSheet="0"/>
-  </oneCellAnchor>
-</wsDr>
-</file>
-
-<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>1</col>
@@ -1616,9 +1646,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+          <c:chart r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -1946,7 +1976,7 @@
       </c>
       <c r="C6" s="151" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>Vinicius Mota</t>
         </is>
       </c>
       <c r="D6" s="146" t="n"/>
@@ -1954,8 +1984,10 @@
       <c r="F6" s="146" t="n"/>
       <c r="G6" s="146" t="n"/>
       <c r="H6" s="147" t="n"/>
-      <c r="I6" s="9" t="b">
-        <v>0</v>
+      <c r="I6" s="178" t="inlineStr">
+        <is>
+          <t>   </t>
+        </is>
       </c>
       <c r="J6" s="21" t="inlineStr">
         <is>
@@ -1979,8 +2011,10 @@
       <c r="F7" s="146" t="n"/>
       <c r="G7" s="146" t="n"/>
       <c r="H7" s="147" t="n"/>
-      <c r="I7" s="9" t="b">
-        <v>0</v>
+      <c r="I7" s="178" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
       </c>
       <c r="J7" s="21" t="inlineStr">
         <is>
@@ -2113,15 +2147,19 @@
     </row>
     <row r="13" ht="20" customHeight="1" s="119">
       <c r="A13" s="7" t="n"/>
-      <c r="B13" s="155" t="inlineStr"/>
-      <c r="C13" s="146" t="n"/>
-      <c r="D13" s="146" t="n"/>
-      <c r="E13" s="146" t="n"/>
-      <c r="F13" s="146" t="n"/>
-      <c r="G13" s="146" t="n"/>
-      <c r="H13" s="146" t="n"/>
-      <c r="I13" s="146" t="n"/>
-      <c r="J13" s="147" t="n"/>
+      <c r="B13" s="181" t="inlineStr">
+        <is>
+          <t>SISTEMA DE GESTÃO DA QUALIDADE</t>
+        </is>
+      </c>
+      <c r="C13" s="183" t="n"/>
+      <c r="D13" s="183" t="n"/>
+      <c r="E13" s="183" t="n"/>
+      <c r="F13" s="183" t="n"/>
+      <c r="G13" s="183" t="n"/>
+      <c r="H13" s="183" t="n"/>
+      <c r="I13" s="183" t="n"/>
+      <c r="J13" s="184" t="n"/>
       <c r="K13" s="17">
         <f>COUNTIF(D14:D24,"X")</f>
         <v/>
@@ -2153,7 +2191,7 @@
       <c r="G14" s="158" t="inlineStr"/>
       <c r="H14" s="157" t="inlineStr"/>
       <c r="I14" s="157" t="inlineStr"/>
-      <c r="J14" s="147" t="n"/>
+      <c r="J14" s="180" t="n"/>
       <c r="K14" s="23">
         <f>(K13)/(K13+L13+M13)</f>
         <v/>
@@ -2195,7 +2233,7 @@
         </is>
       </c>
       <c r="I15" s="157" t="inlineStr"/>
-      <c r="J15" s="147" t="n"/>
+      <c r="J15" s="180" t="n"/>
       <c r="K15" s="26" t="n"/>
       <c r="L15" s="26" t="n"/>
       <c r="M15" s="26" t="n"/>
@@ -2229,7 +2267,7 @@
         </is>
       </c>
       <c r="I16" s="157" t="inlineStr"/>
-      <c r="J16" s="147" t="n"/>
+      <c r="J16" s="180" t="n"/>
       <c r="K16" s="26" t="n"/>
       <c r="L16" s="26" t="n"/>
       <c r="M16" s="26" t="n"/>
@@ -2262,7 +2300,7 @@
         </is>
       </c>
       <c r="I17" s="157" t="inlineStr"/>
-      <c r="J17" s="147" t="n"/>
+      <c r="J17" s="180" t="n"/>
       <c r="K17" s="26" t="n"/>
       <c r="L17" s="26" t="n"/>
       <c r="M17" s="26" t="n"/>
@@ -2294,7 +2332,7 @@
         </is>
       </c>
       <c r="I18" s="157" t="inlineStr"/>
-      <c r="J18" s="147" t="n"/>
+      <c r="J18" s="180" t="n"/>
       <c r="K18" s="26" t="n"/>
       <c r="L18" s="26" t="n"/>
       <c r="M18" s="26" t="n"/>
@@ -2325,7 +2363,7 @@
         </is>
       </c>
       <c r="I19" s="157" t="inlineStr"/>
-      <c r="J19" s="147" t="n"/>
+      <c r="J19" s="180" t="n"/>
       <c r="K19" s="26" t="n"/>
       <c r="L19" s="26" t="n"/>
       <c r="M19" s="26" t="n"/>
@@ -2356,7 +2394,7 @@
         </is>
       </c>
       <c r="I20" s="157" t="inlineStr"/>
-      <c r="J20" s="147" t="n"/>
+      <c r="J20" s="180" t="n"/>
       <c r="K20" s="26" t="n"/>
       <c r="L20" s="26" t="n"/>
       <c r="M20" s="26" t="n"/>
@@ -2379,7 +2417,7 @@
       <c r="G21" s="158" t="inlineStr"/>
       <c r="H21" s="157" t="inlineStr"/>
       <c r="I21" s="157" t="inlineStr"/>
-      <c r="J21" s="147" t="n"/>
+      <c r="J21" s="180" t="n"/>
       <c r="K21" s="26" t="n"/>
       <c r="L21" s="26" t="n"/>
       <c r="M21" s="26" t="n"/>
@@ -2413,7 +2451,7 @@
         </is>
       </c>
       <c r="I22" s="157" t="inlineStr"/>
-      <c r="J22" s="147" t="n"/>
+      <c r="J22" s="180" t="n"/>
       <c r="K22" s="26" t="n"/>
       <c r="L22" s="26" t="n"/>
       <c r="M22" s="26" t="n"/>
@@ -2444,7 +2482,7 @@
         </is>
       </c>
       <c r="I23" s="157" t="inlineStr"/>
-      <c r="J23" s="147" t="n"/>
+      <c r="J23" s="180" t="n"/>
       <c r="K23" s="26" t="n"/>
       <c r="L23" s="26" t="n"/>
       <c r="M23" s="26" t="n"/>
@@ -2477,26 +2515,26 @@
         </is>
       </c>
       <c r="I24" s="157" t="inlineStr"/>
-      <c r="J24" s="147" t="n"/>
+      <c r="J24" s="180" t="n"/>
       <c r="K24" s="26" t="n"/>
       <c r="L24" s="26" t="n"/>
       <c r="M24" s="26" t="n"/>
     </row>
     <row r="25" ht="32" customHeight="1" s="119">
       <c r="A25" s="29" t="n"/>
-      <c r="B25" s="155" t="inlineStr">
-        <is>
-          <t>[OBS com Correção] Disponibilizar para os postos de conferência.</t>
-        </is>
-      </c>
-      <c r="C25" s="146" t="n"/>
-      <c r="D25" s="146" t="n"/>
-      <c r="E25" s="146" t="n"/>
-      <c r="F25" s="146" t="n"/>
-      <c r="G25" s="146" t="n"/>
-      <c r="H25" s="146" t="n"/>
-      <c r="I25" s="146" t="n"/>
-      <c r="J25" s="147" t="n"/>
+      <c r="B25" s="181" t="inlineStr">
+        <is>
+          <t>RESPONSABILIDADE DA DIREÇÃO</t>
+        </is>
+      </c>
+      <c r="C25" s="183" t="n"/>
+      <c r="D25" s="183" t="n"/>
+      <c r="E25" s="183" t="n"/>
+      <c r="F25" s="183" t="n"/>
+      <c r="G25" s="183" t="n"/>
+      <c r="H25" s="183" t="n"/>
+      <c r="I25" s="183" t="n"/>
+      <c r="J25" s="184" t="n"/>
       <c r="K25" s="17">
         <f>COUNTIF(D26:D36,"X")</f>
         <v/>
@@ -2539,7 +2577,7 @@
         </is>
       </c>
       <c r="I26" s="157" t="inlineStr"/>
-      <c r="J26" s="147" t="n"/>
+      <c r="J26" s="180" t="n"/>
       <c r="K26" s="23">
         <f>(K25)/(K25+L25+M25)</f>
         <v/>
@@ -2571,7 +2609,7 @@
       <c r="G27" s="158" t="inlineStr"/>
       <c r="H27" s="157" t="inlineStr"/>
       <c r="I27" s="157" t="inlineStr"/>
-      <c r="J27" s="147" t="n"/>
+      <c r="J27" s="180" t="n"/>
       <c r="K27" s="26" t="n"/>
       <c r="L27" s="26" t="n"/>
       <c r="M27" s="26" t="n"/>
@@ -2624,7 +2662,7 @@
         </is>
       </c>
       <c r="I28" s="157" t="inlineStr"/>
-      <c r="J28" s="147" t="n"/>
+      <c r="J28" s="180" t="n"/>
       <c r="K28" s="26" t="n"/>
       <c r="L28" s="26" t="n"/>
       <c r="M28" s="26" t="n"/>
@@ -2657,7 +2695,7 @@
         </is>
       </c>
       <c r="I29" s="157" t="inlineStr"/>
-      <c r="J29" s="147" t="n"/>
+      <c r="J29" s="180" t="n"/>
       <c r="K29" s="26" t="n"/>
       <c r="L29" s="26" t="n"/>
       <c r="M29" s="26" t="n"/>
@@ -2688,7 +2726,7 @@
         </is>
       </c>
       <c r="I30" s="157" t="inlineStr"/>
-      <c r="J30" s="147" t="n"/>
+      <c r="J30" s="180" t="n"/>
       <c r="K30" s="26" t="n"/>
       <c r="L30" s="26" t="n"/>
       <c r="M30" s="26" t="n"/>
@@ -2711,7 +2749,7 @@
       <c r="G31" s="158" t="inlineStr"/>
       <c r="H31" s="157" t="inlineStr"/>
       <c r="I31" s="157" t="inlineStr"/>
-      <c r="J31" s="147" t="n"/>
+      <c r="J31" s="180" t="n"/>
       <c r="K31" s="26" t="n"/>
       <c r="L31" s="26" t="n"/>
       <c r="M31" s="26" t="n"/>
@@ -2743,7 +2781,7 @@
         </is>
       </c>
       <c r="I32" s="157" t="inlineStr"/>
-      <c r="J32" s="147" t="n"/>
+      <c r="J32" s="180" t="n"/>
       <c r="K32" s="26" t="n"/>
       <c r="L32" s="26" t="n"/>
       <c r="M32" s="26" t="n"/>
@@ -2777,7 +2815,7 @@
         </is>
       </c>
       <c r="I33" s="157" t="inlineStr"/>
-      <c r="J33" s="147" t="n"/>
+      <c r="J33" s="180" t="n"/>
       <c r="K33" s="26" t="n"/>
       <c r="L33" s="26" t="n"/>
       <c r="M33" s="26" t="n"/>
@@ -2800,7 +2838,7 @@
       <c r="G34" s="158" t="inlineStr"/>
       <c r="H34" s="157" t="inlineStr"/>
       <c r="I34" s="157" t="inlineStr"/>
-      <c r="J34" s="147" t="n"/>
+      <c r="J34" s="180" t="n"/>
       <c r="K34" s="26" t="n"/>
       <c r="L34" s="26" t="n"/>
       <c r="M34" s="26" t="n"/>
@@ -2831,7 +2869,7 @@
         </is>
       </c>
       <c r="I35" s="157" t="inlineStr"/>
-      <c r="J35" s="147" t="n"/>
+      <c r="J35" s="180" t="n"/>
       <c r="K35" s="26" t="n"/>
       <c r="L35" s="26" t="n"/>
       <c r="M35" s="26" t="n"/>
@@ -2862,22 +2900,26 @@
         </is>
       </c>
       <c r="I36" s="157" t="inlineStr"/>
-      <c r="J36" s="147" t="n"/>
+      <c r="J36" s="180" t="n"/>
       <c r="K36" s="26" t="n"/>
       <c r="L36" s="26" t="n"/>
       <c r="M36" s="26" t="n"/>
     </row>
     <row r="37" ht="48" customHeight="1" s="119">
       <c r="A37" s="29" t="n"/>
-      <c r="B37" s="155" t="inlineStr"/>
-      <c r="C37" s="146" t="n"/>
-      <c r="D37" s="146" t="n"/>
-      <c r="E37" s="146" t="n"/>
-      <c r="F37" s="146" t="n"/>
-      <c r="G37" s="146" t="n"/>
-      <c r="H37" s="146" t="n"/>
-      <c r="I37" s="146" t="n"/>
-      <c r="J37" s="147" t="n"/>
+      <c r="B37" s="181" t="inlineStr">
+        <is>
+          <t>GESTÃO DE RECURSOS</t>
+        </is>
+      </c>
+      <c r="C37" s="183" t="n"/>
+      <c r="D37" s="183" t="n"/>
+      <c r="E37" s="183" t="n"/>
+      <c r="F37" s="183" t="n"/>
+      <c r="G37" s="183" t="n"/>
+      <c r="H37" s="183" t="n"/>
+      <c r="I37" s="183" t="n"/>
+      <c r="J37" s="184" t="n"/>
       <c r="K37" s="17">
         <f>COUNTIF(D38:D42,"X")</f>
         <v/>
@@ -2909,7 +2951,7 @@
       <c r="G38" s="158" t="inlineStr"/>
       <c r="H38" s="157" t="inlineStr"/>
       <c r="I38" s="157" t="inlineStr"/>
-      <c r="J38" s="147" t="n"/>
+      <c r="J38" s="180" t="n"/>
       <c r="K38" s="23">
         <f>(K37)/(K37+L37+M37)</f>
         <v/>
@@ -2951,7 +2993,7 @@
         </is>
       </c>
       <c r="I39" s="157" t="inlineStr"/>
-      <c r="J39" s="147" t="n"/>
+      <c r="J39" s="180" t="n"/>
       <c r="K39" s="26" t="n"/>
       <c r="L39" s="26" t="n"/>
       <c r="M39" s="26" t="n"/>
@@ -2984,7 +3026,7 @@
         </is>
       </c>
       <c r="I40" s="157" t="inlineStr"/>
-      <c r="J40" s="147" t="n"/>
+      <c r="J40" s="180" t="n"/>
       <c r="K40" s="26" t="n"/>
       <c r="L40" s="26" t="n"/>
       <c r="M40" s="26" t="n"/>
@@ -3017,7 +3059,7 @@
         </is>
       </c>
       <c r="I41" s="157" t="inlineStr"/>
-      <c r="J41" s="147" t="n"/>
+      <c r="J41" s="180" t="n"/>
       <c r="K41" s="26" t="n"/>
       <c r="L41" s="26" t="n"/>
       <c r="M41" s="26" t="n"/>
@@ -3040,22 +3082,26 @@
       <c r="G42" s="158" t="inlineStr"/>
       <c r="H42" s="157" t="inlineStr"/>
       <c r="I42" s="157" t="inlineStr"/>
-      <c r="J42" s="147" t="n"/>
+      <c r="J42" s="180" t="n"/>
       <c r="K42" s="26" t="n"/>
       <c r="L42" s="26" t="n"/>
       <c r="M42" s="26" t="n"/>
     </row>
     <row r="43" ht="48" customHeight="1" s="119">
       <c r="A43" s="29" t="n"/>
-      <c r="B43" s="155" t="inlineStr"/>
-      <c r="C43" s="146" t="n"/>
-      <c r="D43" s="146" t="n"/>
-      <c r="E43" s="146" t="n"/>
-      <c r="F43" s="146" t="n"/>
-      <c r="G43" s="146" t="n"/>
-      <c r="H43" s="146" t="n"/>
-      <c r="I43" s="146" t="n"/>
-      <c r="J43" s="147" t="n"/>
+      <c r="B43" s="181" t="inlineStr">
+        <is>
+          <t>REALIZAÇÃO DE PRODUTO (FABRICAÇÃO)</t>
+        </is>
+      </c>
+      <c r="C43" s="183" t="n"/>
+      <c r="D43" s="183" t="n"/>
+      <c r="E43" s="183" t="n"/>
+      <c r="F43" s="183" t="n"/>
+      <c r="G43" s="183" t="n"/>
+      <c r="H43" s="183" t="n"/>
+      <c r="I43" s="183" t="n"/>
+      <c r="J43" s="184" t="n"/>
       <c r="K43" s="17">
         <f>COUNTIF(D44:D73,"X")</f>
         <v/>
@@ -3138,7 +3184,7 @@
 [OBS com Correção] Foi observado que há campos sem preenchimento, que requerem atualização.</t>
         </is>
       </c>
-      <c r="J44" s="147" t="n"/>
+      <c r="J44" s="180" t="n"/>
       <c r="K44" s="23">
         <f>(K43)/(K43+L43+M43)</f>
         <v/>
@@ -3178,7 +3224,7 @@
         </is>
       </c>
       <c r="I45" s="157" t="inlineStr"/>
-      <c r="J45" s="147" t="n"/>
+      <c r="J45" s="180" t="n"/>
       <c r="K45" s="26" t="n"/>
       <c r="L45" s="26" t="n"/>
       <c r="M45" s="26" t="n"/>
@@ -3201,7 +3247,7 @@
       <c r="G46" s="158" t="inlineStr"/>
       <c r="H46" s="157" t="inlineStr"/>
       <c r="I46" s="157" t="inlineStr"/>
-      <c r="J46" s="147" t="n"/>
+      <c r="J46" s="180" t="n"/>
       <c r="K46" s="26" t="n"/>
       <c r="L46" s="26" t="n"/>
       <c r="M46" s="26" t="n"/>
@@ -3235,7 +3281,7 @@
         </is>
       </c>
       <c r="I47" s="157" t="inlineStr"/>
-      <c r="J47" s="147" t="n"/>
+      <c r="J47" s="180" t="n"/>
       <c r="K47" s="26" t="n"/>
       <c r="L47" s="26" t="n"/>
       <c r="M47" s="26" t="n"/>
@@ -3289,7 +3335,7 @@
         </is>
       </c>
       <c r="I48" s="157" t="inlineStr"/>
-      <c r="J48" s="147" t="n"/>
+      <c r="J48" s="180" t="n"/>
       <c r="K48" s="26" t="n"/>
       <c r="L48" s="26" t="n"/>
       <c r="M48" s="26" t="n"/>
@@ -3312,7 +3358,7 @@
       <c r="G49" s="158" t="inlineStr"/>
       <c r="H49" s="157" t="inlineStr"/>
       <c r="I49" s="157" t="inlineStr"/>
-      <c r="J49" s="147" t="n"/>
+      <c r="J49" s="180" t="n"/>
       <c r="K49" s="26" t="n"/>
       <c r="L49" s="26" t="n"/>
       <c r="M49" s="26" t="n"/>
@@ -3344,7 +3390,7 @@
         </is>
       </c>
       <c r="I50" s="157" t="inlineStr"/>
-      <c r="J50" s="147" t="n"/>
+      <c r="J50" s="180" t="n"/>
       <c r="K50" s="26" t="n"/>
       <c r="L50" s="26" t="n"/>
       <c r="M50" s="26" t="n"/>
@@ -3367,7 +3413,7 @@
       <c r="G51" s="158" t="inlineStr"/>
       <c r="H51" s="157" t="inlineStr"/>
       <c r="I51" s="157" t="inlineStr"/>
-      <c r="J51" s="147" t="n"/>
+      <c r="J51" s="180" t="n"/>
       <c r="K51" s="26" t="n"/>
       <c r="L51" s="26" t="n"/>
       <c r="M51" s="26" t="n"/>
@@ -3402,7 +3448,7 @@
         </is>
       </c>
       <c r="I52" s="157" t="inlineStr"/>
-      <c r="J52" s="147" t="n"/>
+      <c r="J52" s="180" t="n"/>
       <c r="K52" s="26" t="n"/>
       <c r="L52" s="26" t="n"/>
       <c r="M52" s="26" t="n"/>
@@ -3438,7 +3484,7 @@
         </is>
       </c>
       <c r="I53" s="157" t="inlineStr"/>
-      <c r="J53" s="147" t="n"/>
+      <c r="J53" s="180" t="n"/>
       <c r="K53" s="26" t="n"/>
       <c r="L53" s="26" t="n"/>
       <c r="M53" s="26" t="n"/>
@@ -3474,7 +3520,7 @@
         </is>
       </c>
       <c r="I54" s="157" t="inlineStr"/>
-      <c r="J54" s="147" t="n"/>
+      <c r="J54" s="180" t="n"/>
       <c r="K54" s="26" t="n"/>
       <c r="L54" s="26" t="n"/>
       <c r="M54" s="26" t="n"/>
@@ -3497,7 +3543,7 @@
       <c r="G55" s="158" t="inlineStr"/>
       <c r="H55" s="157" t="inlineStr"/>
       <c r="I55" s="157" t="inlineStr"/>
-      <c r="J55" s="147" t="n"/>
+      <c r="J55" s="180" t="n"/>
       <c r="K55" s="26" t="n"/>
       <c r="L55" s="26" t="n"/>
       <c r="M55" s="26" t="n"/>
@@ -3524,7 +3570,7 @@
       <c r="G56" s="158" t="inlineStr"/>
       <c r="H56" s="157" t="inlineStr"/>
       <c r="I56" s="157" t="inlineStr"/>
-      <c r="J56" s="147" t="n"/>
+      <c r="J56" s="180" t="n"/>
       <c r="K56" s="26" t="n"/>
       <c r="L56" s="26" t="n"/>
       <c r="M56" s="26" t="n"/>
@@ -3551,7 +3597,7 @@
       <c r="G57" s="158" t="inlineStr"/>
       <c r="H57" s="157" t="inlineStr"/>
       <c r="I57" s="157" t="inlineStr"/>
-      <c r="J57" s="147" t="n"/>
+      <c r="J57" s="180" t="n"/>
       <c r="K57" s="26" t="n"/>
       <c r="L57" s="26" t="n"/>
       <c r="M57" s="26" t="n"/>
@@ -3578,7 +3624,7 @@
       <c r="G58" s="158" t="inlineStr"/>
       <c r="H58" s="157" t="inlineStr"/>
       <c r="I58" s="157" t="inlineStr"/>
-      <c r="J58" s="147" t="n"/>
+      <c r="J58" s="180" t="n"/>
       <c r="K58" s="26" t="n"/>
       <c r="L58" s="26" t="n"/>
       <c r="M58" s="26" t="n"/>
@@ -3605,7 +3651,7 @@
       <c r="G59" s="158" t="inlineStr"/>
       <c r="H59" s="157" t="inlineStr"/>
       <c r="I59" s="157" t="inlineStr"/>
-      <c r="J59" s="147" t="n"/>
+      <c r="J59" s="180" t="n"/>
       <c r="K59" s="26" t="n"/>
       <c r="L59" s="26" t="n"/>
       <c r="M59" s="26" t="n"/>
@@ -3632,7 +3678,7 @@
       <c r="G60" s="158" t="inlineStr"/>
       <c r="H60" s="157" t="inlineStr"/>
       <c r="I60" s="157" t="inlineStr"/>
-      <c r="J60" s="147" t="n"/>
+      <c r="J60" s="180" t="n"/>
       <c r="K60" s="26" t="n"/>
       <c r="L60" s="26" t="n"/>
       <c r="M60" s="26" t="n"/>
@@ -3659,7 +3705,7 @@
       <c r="G61" s="158" t="inlineStr"/>
       <c r="H61" s="157" t="inlineStr"/>
       <c r="I61" s="157" t="inlineStr"/>
-      <c r="J61" s="147" t="n"/>
+      <c r="J61" s="180" t="n"/>
       <c r="K61" s="26" t="n"/>
       <c r="L61" s="26" t="n"/>
       <c r="M61" s="26" t="n"/>
@@ -3686,7 +3732,7 @@
       <c r="G62" s="158" t="inlineStr"/>
       <c r="H62" s="157" t="inlineStr"/>
       <c r="I62" s="157" t="inlineStr"/>
-      <c r="J62" s="147" t="n"/>
+      <c r="J62" s="180" t="n"/>
       <c r="K62" s="26" t="n"/>
       <c r="L62" s="26" t="n"/>
       <c r="M62" s="26" t="n"/>
@@ -3713,7 +3759,7 @@
       <c r="G63" s="158" t="inlineStr"/>
       <c r="H63" s="157" t="inlineStr"/>
       <c r="I63" s="157" t="inlineStr"/>
-      <c r="J63" s="147" t="n"/>
+      <c r="J63" s="180" t="n"/>
       <c r="K63" s="26" t="n"/>
       <c r="L63" s="26" t="n"/>
       <c r="M63" s="26" t="n"/>
@@ -3740,7 +3786,7 @@
       <c r="G64" s="158" t="inlineStr"/>
       <c r="H64" s="157" t="inlineStr"/>
       <c r="I64" s="157" t="inlineStr"/>
-      <c r="J64" s="147" t="n"/>
+      <c r="J64" s="180" t="n"/>
       <c r="K64" s="26" t="n"/>
       <c r="L64" s="26" t="n"/>
       <c r="M64" s="26" t="n"/>
@@ -3767,7 +3813,7 @@
       <c r="G65" s="158" t="inlineStr"/>
       <c r="H65" s="157" t="inlineStr"/>
       <c r="I65" s="157" t="inlineStr"/>
-      <c r="J65" s="147" t="n"/>
+      <c r="J65" s="180" t="n"/>
       <c r="K65" s="26" t="n"/>
       <c r="L65" s="26" t="n"/>
       <c r="M65" s="26" t="n"/>
@@ -3790,7 +3836,7 @@
       <c r="G66" s="158" t="inlineStr"/>
       <c r="H66" s="157" t="inlineStr"/>
       <c r="I66" s="157" t="inlineStr"/>
-      <c r="J66" s="147" t="n"/>
+      <c r="J66" s="180" t="n"/>
       <c r="K66" s="26" t="n"/>
       <c r="L66" s="26" t="n"/>
       <c r="M66" s="26" t="n"/>
@@ -3822,7 +3868,7 @@
         </is>
       </c>
       <c r="I67" s="157" t="inlineStr"/>
-      <c r="J67" s="147" t="n"/>
+      <c r="J67" s="180" t="n"/>
       <c r="K67" s="26" t="n"/>
       <c r="L67" s="26" t="n"/>
       <c r="M67" s="26" t="n"/>
@@ -3855,7 +3901,7 @@
         </is>
       </c>
       <c r="I68" s="157" t="inlineStr"/>
-      <c r="J68" s="147" t="n"/>
+      <c r="J68" s="180" t="n"/>
       <c r="K68" s="26" t="n"/>
       <c r="L68" s="26" t="n"/>
       <c r="M68" s="26" t="n"/>
@@ -3889,7 +3935,7 @@
         </is>
       </c>
       <c r="I69" s="157" t="inlineStr"/>
-      <c r="J69" s="147" t="n"/>
+      <c r="J69" s="180" t="n"/>
       <c r="K69" s="26" t="n"/>
       <c r="L69" s="26" t="n"/>
       <c r="M69" s="26" t="n"/>
@@ -3912,7 +3958,7 @@
       <c r="G70" s="158" t="inlineStr"/>
       <c r="H70" s="157" t="inlineStr"/>
       <c r="I70" s="157" t="inlineStr"/>
-      <c r="J70" s="147" t="n"/>
+      <c r="J70" s="180" t="n"/>
       <c r="K70" s="26" t="n"/>
       <c r="L70" s="26" t="n"/>
       <c r="M70" s="26" t="n"/>
@@ -3953,7 +3999,7 @@
         </is>
       </c>
       <c r="I71" s="157" t="inlineStr"/>
-      <c r="J71" s="147" t="n"/>
+      <c r="J71" s="180" t="n"/>
       <c r="K71" s="26" t="n"/>
       <c r="L71" s="26" t="n"/>
       <c r="M71" s="26" t="n"/>
@@ -3985,7 +4031,7 @@
         </is>
       </c>
       <c r="I72" s="157" t="inlineStr"/>
-      <c r="J72" s="147" t="n"/>
+      <c r="J72" s="180" t="n"/>
       <c r="K72" s="26" t="n"/>
       <c r="L72" s="26" t="n"/>
       <c r="M72" s="26" t="n"/>
@@ -4012,22 +4058,26 @@
       <c r="G73" s="158" t="inlineStr"/>
       <c r="H73" s="157" t="inlineStr"/>
       <c r="I73" s="157" t="inlineStr"/>
-      <c r="J73" s="147" t="n"/>
+      <c r="J73" s="180" t="n"/>
       <c r="K73" s="26" t="n"/>
       <c r="L73" s="26" t="n"/>
       <c r="M73" s="26" t="n"/>
     </row>
     <row r="74" ht="20" customHeight="1" s="119">
       <c r="A74" s="29" t="n"/>
-      <c r="B74" s="155" t="inlineStr"/>
-      <c r="C74" s="146" t="n"/>
-      <c r="D74" s="146" t="n"/>
-      <c r="E74" s="146" t="n"/>
-      <c r="F74" s="146" t="n"/>
-      <c r="G74" s="146" t="n"/>
-      <c r="H74" s="146" t="n"/>
-      <c r="I74" s="146" t="n"/>
-      <c r="J74" s="147" t="n"/>
+      <c r="B74" s="181" t="inlineStr">
+        <is>
+          <t>MEDIÇÃO, ANÁLISE E MELHORIA</t>
+        </is>
+      </c>
+      <c r="C74" s="183" t="n"/>
+      <c r="D74" s="183" t="n"/>
+      <c r="E74" s="183" t="n"/>
+      <c r="F74" s="183" t="n"/>
+      <c r="G74" s="183" t="n"/>
+      <c r="H74" s="183" t="n"/>
+      <c r="I74" s="183" t="n"/>
+      <c r="J74" s="184" t="n"/>
       <c r="K74" s="17">
         <f>COUNTIF(D75:D89,"X")</f>
         <v/>
@@ -4063,7 +4113,7 @@
       <c r="G75" s="158" t="inlineStr"/>
       <c r="H75" s="157" t="inlineStr"/>
       <c r="I75" s="157" t="inlineStr"/>
-      <c r="J75" s="147" t="n"/>
+      <c r="J75" s="180" t="n"/>
       <c r="K75" s="23">
         <f>(K74)/(K74+L74+M74)</f>
         <v/>
@@ -4104,7 +4154,7 @@
         </is>
       </c>
       <c r="I76" s="157" t="inlineStr"/>
-      <c r="J76" s="147" t="n"/>
+      <c r="J76" s="180" t="n"/>
       <c r="K76" s="26" t="n"/>
       <c r="L76" s="26" t="n"/>
       <c r="M76" s="26" t="n"/>
@@ -4131,7 +4181,7 @@
       <c r="G77" s="158" t="inlineStr"/>
       <c r="H77" s="157" t="inlineStr"/>
       <c r="I77" s="157" t="inlineStr"/>
-      <c r="J77" s="147" t="n"/>
+      <c r="J77" s="180" t="n"/>
       <c r="K77" s="26" t="n"/>
       <c r="L77" s="26" t="n"/>
       <c r="M77" s="26" t="n"/>
@@ -4165,7 +4215,7 @@
         </is>
       </c>
       <c r="I78" s="157" t="inlineStr"/>
-      <c r="J78" s="147" t="n"/>
+      <c r="J78" s="180" t="n"/>
       <c r="K78" s="26" t="n"/>
       <c r="L78" s="26" t="n"/>
       <c r="M78" s="26" t="n"/>
@@ -4188,7 +4238,7 @@
       <c r="G79" s="158" t="inlineStr"/>
       <c r="H79" s="157" t="inlineStr"/>
       <c r="I79" s="157" t="inlineStr"/>
-      <c r="J79" s="147" t="n"/>
+      <c r="J79" s="180" t="n"/>
       <c r="K79" s="26" t="n"/>
       <c r="L79" s="26" t="n"/>
       <c r="M79" s="26" t="n"/>
@@ -4221,7 +4271,7 @@
         </is>
       </c>
       <c r="I80" s="157" t="inlineStr"/>
-      <c r="J80" s="147" t="n"/>
+      <c r="J80" s="180" t="n"/>
       <c r="K80" s="26" t="n"/>
       <c r="L80" s="26" t="n"/>
       <c r="M80" s="26" t="n"/>
@@ -4248,7 +4298,7 @@
       <c r="G81" s="158" t="inlineStr"/>
       <c r="H81" s="157" t="inlineStr"/>
       <c r="I81" s="157" t="inlineStr"/>
-      <c r="J81" s="147" t="n"/>
+      <c r="J81" s="180" t="n"/>
       <c r="K81" s="26" t="n"/>
       <c r="L81" s="26" t="n"/>
       <c r="M81" s="26" t="n"/>
@@ -4284,7 +4334,7 @@
         </is>
       </c>
       <c r="I82" s="157" t="inlineStr"/>
-      <c r="J82" s="147" t="n"/>
+      <c r="J82" s="180" t="n"/>
       <c r="K82" s="26" t="n"/>
       <c r="L82" s="26" t="n"/>
       <c r="M82" s="26" t="n"/>
@@ -4316,7 +4366,7 @@
         </is>
       </c>
       <c r="I83" s="157" t="inlineStr"/>
-      <c r="J83" s="147" t="n"/>
+      <c r="J83" s="180" t="n"/>
       <c r="K83" s="26" t="n"/>
       <c r="L83" s="26" t="n"/>
       <c r="M83" s="26" t="n"/>
@@ -4365,7 +4415,7 @@
         </is>
       </c>
       <c r="I84" s="157" t="inlineStr"/>
-      <c r="J84" s="147" t="n"/>
+      <c r="J84" s="180" t="n"/>
       <c r="K84" s="26" t="n"/>
       <c r="L84" s="26" t="n"/>
       <c r="M84" s="26" t="n"/>
@@ -4388,7 +4438,7 @@
       <c r="G85" s="158" t="inlineStr"/>
       <c r="H85" s="157" t="inlineStr"/>
       <c r="I85" s="157" t="inlineStr"/>
-      <c r="J85" s="147" t="n"/>
+      <c r="J85" s="180" t="n"/>
       <c r="K85" s="26" t="n"/>
       <c r="L85" s="26" t="n"/>
       <c r="M85" s="26" t="n"/>
@@ -4431,7 +4481,7 @@
         </is>
       </c>
       <c r="I86" s="157" t="inlineStr"/>
-      <c r="J86" s="147" t="n"/>
+      <c r="J86" s="180" t="n"/>
       <c r="K86" s="26" t="n"/>
       <c r="L86" s="26" t="n"/>
       <c r="M86" s="26" t="n"/>
@@ -4454,7 +4504,7 @@
       <c r="G87" s="158" t="inlineStr"/>
       <c r="H87" s="157" t="inlineStr"/>
       <c r="I87" s="157" t="inlineStr"/>
-      <c r="J87" s="147" t="n"/>
+      <c r="J87" s="180" t="n"/>
       <c r="K87" s="26" t="n"/>
       <c r="L87" s="26" t="n"/>
       <c r="M87" s="26" t="n"/>
@@ -4490,7 +4540,7 @@
         </is>
       </c>
       <c r="I88" s="157" t="inlineStr"/>
-      <c r="J88" s="147" t="n"/>
+      <c r="J88" s="180" t="n"/>
       <c r="K88" s="26" t="n"/>
       <c r="L88" s="26" t="n"/>
       <c r="M88" s="26" t="n"/>
@@ -4526,7 +4576,7 @@
         </is>
       </c>
       <c r="I89" s="157" t="inlineStr"/>
-      <c r="J89" s="147" t="n"/>
+      <c r="J89" s="180" t="n"/>
       <c r="K89" s="26" t="n"/>
       <c r="L89" s="26" t="n"/>
       <c r="M89" s="26" t="n"/>
@@ -4543,15 +4593,17 @@
           <t>Notificação às autoridades regulatórias</t>
         </is>
       </c>
-      <c r="D90" s="162" t="inlineStr">
+      <c r="D90" s="182" t="inlineStr">
         <is>
           <t>X</t>
         </is>
       </c>
-      <c r="E90" s="163" t="inlineStr"/>
-      <c r="F90" s="157" t="inlineStr">
-        <is>
-          <t>• [Conforme] PSQ.022.R5: Não Conformidade - Ações Corretivas e Preventivas: A organização deve realizar o acompanhamento de todas as soluções de problemas e oportunidades de melhorias criadas para que o sistema de qualidade esteja em constante melhoria dos seus processos. Neste  sentido,  é  obrigatório  inserir  todos  os  registros  relacionados  no  Controle  Anual  de  Registros: Plano de Ação, RNC, 8D, Gestão de Mudança e Revisão Gerencial.
+      <c r="E90" s="163" t="n"/>
+      <c r="F90" s="157" t="n"/>
+      <c r="G90" s="185" t="n"/>
+      <c r="H90" s="157" t="inlineStr">
+        <is>
+          <t>• [Conforme] PSQ.022.R5: Não Conformidade - Ações Corretivas e Preventivas: A organização deve realizar o acompanhamento de todas as soluções de problemas e oportunidades de melhorias criadas para que o sistema de qualidade esteja em constante melhoria dos seus processos. Neste sentido, é obrigatório inserir todos os registros relacionados no Controle Anual de Registros: Plano de Ação, RNC, 8D, Gestão de Mudança e Revisão Gerencial.
 • [Conforme] POP.1057.R0: Manual Operacional - Comunicação com o Cliente - Visolab: 2. RECLAMAÇÕES: 
 2.1 Recebimento de Reclamações 
 2.2 Tratativa das Reclamações:
@@ -4563,10 +4615,8 @@
 4. PESQUISA ANUAL DE SATISFAÇÃO</t>
         </is>
       </c>
-      <c r="G90" s="149" t="n"/>
-      <c r="H90" s="149" t="n"/>
       <c r="I90" s="157" t="inlineStr"/>
-      <c r="J90" s="53" t="n"/>
+      <c r="J90" s="185" t="n"/>
       <c r="K90" s="5" t="n"/>
       <c r="L90" s="5" t="n"/>
       <c r="M90" s="5" t="n"/>
@@ -4583,13 +4633,15 @@
           <t>Auditoria interna</t>
         </is>
       </c>
-      <c r="D91" s="162" t="inlineStr">
+      <c r="D91" s="182" t="inlineStr">
         <is>
           <t>X</t>
         </is>
       </c>
-      <c r="E91" s="163" t="inlineStr"/>
-      <c r="F91" s="157" t="inlineStr">
+      <c r="E91" s="163" t="n"/>
+      <c r="F91" s="157" t="n"/>
+      <c r="G91" s="185" t="n"/>
+      <c r="H91" s="157" t="inlineStr">
         <is>
           <t>• [Conforme] PSQ.024.R3: Auditoria: FOR.140: Relatório de Auditoria Interna, 
 FOR.123: Agenda de Auditoria, 
@@ -4598,7 +4650,7 @@
         </is>
       </c>
       <c r="I91" s="157" t="inlineStr"/>
-      <c r="J91" s="53" t="n"/>
+      <c r="J91" s="185" t="n"/>
       <c r="K91" s="5" t="n"/>
       <c r="L91" s="5" t="n"/>
       <c r="M91" s="5" t="n"/>
@@ -4615,20 +4667,22 @@
           <t>Monitoramento e medição de processos</t>
         </is>
       </c>
-      <c r="D92" s="162" t="inlineStr">
+      <c r="D92" s="182" t="inlineStr">
         <is>
           <t>X</t>
         </is>
       </c>
-      <c r="E92" s="163" t="inlineStr"/>
-      <c r="F92" s="157" t="inlineStr">
+      <c r="E92" s="163" t="n"/>
+      <c r="F92" s="157" t="n"/>
+      <c r="G92" s="185" t="n"/>
+      <c r="H92" s="157" t="inlineStr">
         <is>
           <t>• [Conforme] Evidências / Documentos Registrados: MAQ.002.R10 - Manual da Qualidade:
 - Objetivos da Qualidade</t>
         </is>
       </c>
       <c r="I92" s="157" t="inlineStr"/>
-      <c r="J92" s="53" t="n"/>
+      <c r="J92" s="185" t="n"/>
       <c r="K92" s="5" t="n"/>
       <c r="L92" s="5" t="n"/>
       <c r="M92" s="5" t="n"/>
@@ -4645,13 +4699,15 @@
           <t>Monitoramento e medição de produto</t>
         </is>
       </c>
-      <c r="D93" s="162" t="inlineStr">
+      <c r="D93" s="182" t="inlineStr">
         <is>
           <t>X</t>
         </is>
       </c>
-      <c r="E93" s="163" t="inlineStr"/>
-      <c r="F93" s="157" t="inlineStr">
+      <c r="E93" s="163" t="n"/>
+      <c r="F93" s="157" t="n"/>
+      <c r="G93" s="185" t="n"/>
+      <c r="H93" s="157" t="inlineStr">
         <is>
           <t>• [Conforme] Evidências / Documentos Registrados: PSQ.018.R2 - Realização de Produto; 
 PSQ.017.R3 - Controle de Documentos e Registros; 
@@ -4671,7 +4727,7 @@
         </is>
       </c>
       <c r="I93" s="157" t="inlineStr"/>
-      <c r="J93" s="53" t="n"/>
+      <c r="J93" s="185" t="n"/>
       <c r="K93" s="5" t="n"/>
       <c r="L93" s="5" t="n"/>
       <c r="M93" s="5" t="n"/>
@@ -5002,7 +5058,6 @@
     <mergeCell ref="I76:J76"/>
     <mergeCell ref="I71:J71"/>
     <mergeCell ref="I66:J66"/>
-    <mergeCell ref="F92:H92"/>
     <mergeCell ref="I18:J18"/>
     <mergeCell ref="I58:J58"/>
     <mergeCell ref="I42:J42"/>
@@ -5021,7 +5076,6 @@
     <mergeCell ref="I86:J86"/>
     <mergeCell ref="I80:J80"/>
     <mergeCell ref="I61:J61"/>
-    <mergeCell ref="F91:H91"/>
     <mergeCell ref="I70:J70"/>
     <mergeCell ref="I57:J57"/>
     <mergeCell ref="B37:J37"/>
@@ -5029,7 +5083,6 @@
     <mergeCell ref="I32:J32"/>
     <mergeCell ref="I72:J72"/>
     <mergeCell ref="I41:J41"/>
-    <mergeCell ref="F93:H93"/>
     <mergeCell ref="I56:J56"/>
     <mergeCell ref="C9:J9"/>
     <mergeCell ref="I24:J24"/>
@@ -5045,7 +5098,6 @@
     <mergeCell ref="B43:J43"/>
     <mergeCell ref="I60:J60"/>
     <mergeCell ref="I45:J45"/>
-    <mergeCell ref="F90:H90"/>
     <mergeCell ref="I47:J47"/>
     <mergeCell ref="I21:J21"/>
     <mergeCell ref="I87:J87"/>
@@ -5062,19 +5114,23 @@
     <mergeCell ref="I50:J50"/>
     <mergeCell ref="I65:J65"/>
     <mergeCell ref="I34:J34"/>
+    <mergeCell ref="I90:J90"/>
     <mergeCell ref="I49:J49"/>
     <mergeCell ref="I27:J27"/>
     <mergeCell ref="I36:J36"/>
+    <mergeCell ref="I91:J91"/>
     <mergeCell ref="I85:J85"/>
     <mergeCell ref="B10:J10"/>
     <mergeCell ref="I75:J75"/>
     <mergeCell ref="I22:J22"/>
     <mergeCell ref="I28:J28"/>
     <mergeCell ref="I53:J53"/>
+    <mergeCell ref="I93:J93"/>
     <mergeCell ref="B74:J74"/>
     <mergeCell ref="C7:H7"/>
     <mergeCell ref="I12:J12"/>
     <mergeCell ref="I68:J68"/>
+    <mergeCell ref="I92:J92"/>
     <mergeCell ref="I55:J55"/>
     <mergeCell ref="I67:J67"/>
     <mergeCell ref="I5:J5"/>
@@ -5109,7 +5165,6 @@
     <brk id="77" min="0" max="12" man="1"/>
     <brk id="84" min="0" max="16383" man="1"/>
   </rowBreaks>
-  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
feat(checklist): preencher tabela de Principais Itens com NCs/OMs na aba Resultados
</commit_message>
<xml_diff>
--- a/Checklist_Auditoria_ISO_13485_2016_3 (1).xlsx
+++ b/Checklist_Auditoria_ISO_13485_2016_3 (1).xlsx
@@ -562,7 +562,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="157">
+  <cellXfs count="159">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -975,6 +975,10 @@
     </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="39" fillId="0" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2076,7 +2080,7 @@
         </is>
       </c>
       <c r="I14" s="142" t="n"/>
-      <c r="J14" s="128" t="n"/>
+      <c r="J14" s="157" t="n"/>
       <c r="K14" s="20">
         <f>(K13)/(K13+L13+M13)</f>
         <v/>
@@ -2124,7 +2128,7 @@
         </is>
       </c>
       <c r="I15" s="142" t="n"/>
-      <c r="J15" s="128" t="n"/>
+      <c r="J15" s="157" t="n"/>
       <c r="K15" s="22" t="n"/>
       <c r="L15" s="22" t="n"/>
       <c r="M15" s="22" t="n"/>
@@ -2155,7 +2159,7 @@
         </is>
       </c>
       <c r="I16" s="142" t="n"/>
-      <c r="J16" s="128" t="n"/>
+      <c r="J16" s="157" t="n"/>
       <c r="K16" s="22" t="n"/>
       <c r="L16" s="22" t="n"/>
       <c r="M16" s="22" t="n"/>
@@ -2186,7 +2190,7 @@
         </is>
       </c>
       <c r="I17" s="142" t="n"/>
-      <c r="J17" s="128" t="n"/>
+      <c r="J17" s="157" t="n"/>
       <c r="K17" s="22" t="n"/>
       <c r="L17" s="22" t="n"/>
       <c r="M17" s="22" t="n"/>
@@ -2218,7 +2222,7 @@
         </is>
       </c>
       <c r="I18" s="142" t="n"/>
-      <c r="J18" s="128" t="n"/>
+      <c r="J18" s="157" t="n"/>
       <c r="K18" s="22" t="n"/>
       <c r="L18" s="22" t="n"/>
       <c r="M18" s="22" t="n"/>
@@ -2250,7 +2254,7 @@
         </is>
       </c>
       <c r="I19" s="142" t="n"/>
-      <c r="J19" s="128" t="n"/>
+      <c r="J19" s="157" t="n"/>
       <c r="K19" s="22" t="n"/>
       <c r="L19" s="22" t="n"/>
       <c r="M19" s="22" t="n"/>
@@ -2282,7 +2286,7 @@
         </is>
       </c>
       <c r="I20" s="142" t="n"/>
-      <c r="J20" s="128" t="n"/>
+      <c r="J20" s="157" t="n"/>
       <c r="K20" s="22" t="n"/>
       <c r="L20" s="22" t="n"/>
       <c r="M20" s="22" t="n"/>
@@ -2316,7 +2320,7 @@
         </is>
       </c>
       <c r="I21" s="142" t="n"/>
-      <c r="J21" s="128" t="n"/>
+      <c r="J21" s="157" t="n"/>
       <c r="K21" s="22" t="n"/>
       <c r="L21" s="22" t="n"/>
       <c r="M21" s="22" t="n"/>
@@ -2348,7 +2352,7 @@
         </is>
       </c>
       <c r="I22" s="142" t="n"/>
-      <c r="J22" s="128" t="n"/>
+      <c r="J22" s="157" t="n"/>
       <c r="K22" s="22" t="n"/>
       <c r="L22" s="22" t="n"/>
       <c r="M22" s="22" t="n"/>
@@ -2379,7 +2383,7 @@
         </is>
       </c>
       <c r="I23" s="142" t="n"/>
-      <c r="J23" s="128" t="n"/>
+      <c r="J23" s="157" t="n"/>
       <c r="K23" s="22" t="n"/>
       <c r="L23" s="22" t="n"/>
       <c r="M23" s="22" t="n"/>
@@ -2410,7 +2414,7 @@
         </is>
       </c>
       <c r="I24" s="142" t="n"/>
-      <c r="J24" s="128" t="n"/>
+      <c r="J24" s="157" t="n"/>
       <c r="K24" s="22" t="n"/>
       <c r="L24" s="22" t="n"/>
       <c r="M24" s="22" t="n"/>
@@ -2472,7 +2476,7 @@
         </is>
       </c>
       <c r="I26" s="142" t="n"/>
-      <c r="J26" s="128" t="n"/>
+      <c r="J26" s="157" t="n"/>
       <c r="K26" s="20">
         <f>(K25)/(K25+L25+M25)</f>
         <v/>
@@ -2513,7 +2517,7 @@
         </is>
       </c>
       <c r="I27" s="142" t="n"/>
-      <c r="J27" s="128" t="n"/>
+      <c r="J27" s="157" t="n"/>
       <c r="K27" s="22" t="n"/>
       <c r="L27" s="22" t="n"/>
       <c r="M27" s="22" t="n"/>
@@ -2545,7 +2549,7 @@
         </is>
       </c>
       <c r="I28" s="142" t="n"/>
-      <c r="J28" s="128" t="n"/>
+      <c r="J28" s="157" t="n"/>
       <c r="K28" s="22" t="n"/>
       <c r="L28" s="22" t="n"/>
       <c r="M28" s="22" t="n"/>
@@ -2577,7 +2581,7 @@
         </is>
       </c>
       <c r="I29" s="142" t="n"/>
-      <c r="J29" s="128" t="n"/>
+      <c r="J29" s="157" t="n"/>
       <c r="K29" s="22" t="n"/>
       <c r="L29" s="22" t="n"/>
       <c r="M29" s="22" t="n"/>
@@ -2610,7 +2614,7 @@
         </is>
       </c>
       <c r="I30" s="142" t="n"/>
-      <c r="J30" s="128" t="n"/>
+      <c r="J30" s="157" t="n"/>
       <c r="K30" s="22" t="n"/>
       <c r="L30" s="22" t="n"/>
       <c r="M30" s="22" t="n"/>
@@ -2642,7 +2646,7 @@
         </is>
       </c>
       <c r="I31" s="142" t="n"/>
-      <c r="J31" s="128" t="n"/>
+      <c r="J31" s="157" t="n"/>
       <c r="K31" s="22" t="n"/>
       <c r="L31" s="22" t="n"/>
       <c r="M31" s="22" t="n"/>
@@ -2673,7 +2677,7 @@
         </is>
       </c>
       <c r="I32" s="142" t="n"/>
-      <c r="J32" s="128" t="n"/>
+      <c r="J32" s="157" t="n"/>
       <c r="K32" s="22" t="n"/>
       <c r="L32" s="22" t="n"/>
       <c r="M32" s="22" t="n"/>
@@ -2704,7 +2708,7 @@
         </is>
       </c>
       <c r="I33" s="142" t="n"/>
-      <c r="J33" s="128" t="n"/>
+      <c r="J33" s="157" t="n"/>
       <c r="K33" s="22" t="n"/>
       <c r="L33" s="22" t="n"/>
       <c r="M33" s="22" t="n"/>
@@ -2735,7 +2739,7 @@
         </is>
       </c>
       <c r="I34" s="142" t="n"/>
-      <c r="J34" s="128" t="n"/>
+      <c r="J34" s="157" t="n"/>
       <c r="K34" s="22" t="n"/>
       <c r="L34" s="22" t="n"/>
       <c r="M34" s="22" t="n"/>
@@ -2766,7 +2770,7 @@
         </is>
       </c>
       <c r="I35" s="155" t="n"/>
-      <c r="J35" s="128" t="n"/>
+      <c r="J35" s="157" t="n"/>
       <c r="K35" s="22" t="n"/>
       <c r="L35" s="22" t="n"/>
       <c r="M35" s="22" t="n"/>
@@ -2797,7 +2801,7 @@
         </is>
       </c>
       <c r="I36" s="155" t="n"/>
-      <c r="J36" s="128" t="n"/>
+      <c r="J36" s="157" t="n"/>
       <c r="K36" s="22" t="n"/>
       <c r="L36" s="22" t="n"/>
       <c r="M36" s="22" t="n"/>
@@ -2856,7 +2860,7 @@
         </is>
       </c>
       <c r="I38" s="142" t="n"/>
-      <c r="J38" s="128" t="n"/>
+      <c r="J38" s="157" t="n"/>
       <c r="K38" s="20">
         <f>(K37)/(K37+L37+M37)</f>
         <v/>
@@ -2896,7 +2900,7 @@
         </is>
       </c>
       <c r="I39" s="142" t="n"/>
-      <c r="J39" s="128" t="n"/>
+      <c r="J39" s="157" t="n"/>
       <c r="K39" s="22" t="n"/>
       <c r="L39" s="22" t="n"/>
       <c r="M39" s="22" t="n"/>
@@ -2927,7 +2931,7 @@
         </is>
       </c>
       <c r="I40" s="142" t="n"/>
-      <c r="J40" s="128" t="n"/>
+      <c r="J40" s="157" t="n"/>
       <c r="K40" s="22" t="n"/>
       <c r="L40" s="22" t="n"/>
       <c r="M40" s="22" t="n"/>
@@ -2958,7 +2962,7 @@
         </is>
       </c>
       <c r="I41" s="142" t="n"/>
-      <c r="J41" s="128" t="n"/>
+      <c r="J41" s="157" t="n"/>
       <c r="K41" s="22" t="n"/>
       <c r="L41" s="22" t="n"/>
       <c r="M41" s="22" t="n"/>
@@ -2989,7 +2993,7 @@
         </is>
       </c>
       <c r="I42" s="155" t="n"/>
-      <c r="J42" s="128" t="n"/>
+      <c r="J42" s="157" t="n"/>
       <c r="K42" s="22" t="n"/>
       <c r="L42" s="22" t="n"/>
       <c r="M42" s="22" t="n"/>
@@ -3048,7 +3052,7 @@
         </is>
       </c>
       <c r="I44" s="155" t="n"/>
-      <c r="J44" s="128" t="n"/>
+      <c r="J44" s="157" t="n"/>
       <c r="K44" s="20">
         <f>(K43)/(K43+L43+M43)</f>
         <v/>
@@ -3088,7 +3092,7 @@
         </is>
       </c>
       <c r="I45" s="155" t="n"/>
-      <c r="J45" s="128" t="n"/>
+      <c r="J45" s="157" t="n"/>
       <c r="K45" s="22" t="n"/>
       <c r="L45" s="22" t="n"/>
       <c r="M45" s="22" t="n"/>
@@ -3119,7 +3123,7 @@
         </is>
       </c>
       <c r="I46" s="155" t="n"/>
-      <c r="J46" s="128" t="n"/>
+      <c r="J46" s="157" t="n"/>
       <c r="K46" s="22" t="n"/>
       <c r="L46" s="22" t="n"/>
       <c r="M46" s="22" t="n"/>
@@ -3150,7 +3154,7 @@
         </is>
       </c>
       <c r="I47" s="155" t="n"/>
-      <c r="J47" s="128" t="n"/>
+      <c r="J47" s="157" t="n"/>
       <c r="K47" s="22" t="n"/>
       <c r="L47" s="22" t="n"/>
       <c r="M47" s="22" t="n"/>
@@ -3181,7 +3185,7 @@
         </is>
       </c>
       <c r="I48" s="155" t="n"/>
-      <c r="J48" s="128" t="n"/>
+      <c r="J48" s="157" t="n"/>
       <c r="K48" s="22" t="n"/>
       <c r="L48" s="22" t="n"/>
       <c r="M48" s="22" t="n"/>
@@ -3212,7 +3216,7 @@
         </is>
       </c>
       <c r="I49" s="155" t="n"/>
-      <c r="J49" s="128" t="n"/>
+      <c r="J49" s="157" t="n"/>
       <c r="K49" s="22" t="n"/>
       <c r="L49" s="22" t="n"/>
       <c r="M49" s="22" t="n"/>
@@ -3243,7 +3247,7 @@
         </is>
       </c>
       <c r="I50" s="155" t="n"/>
-      <c r="J50" s="128" t="n"/>
+      <c r="J50" s="157" t="n"/>
       <c r="K50" s="22" t="n"/>
       <c r="L50" s="22" t="n"/>
       <c r="M50" s="22" t="n"/>
@@ -3274,7 +3278,7 @@
         </is>
       </c>
       <c r="I51" s="155" t="n"/>
-      <c r="J51" s="128" t="n"/>
+      <c r="J51" s="157" t="n"/>
       <c r="K51" s="22" t="n"/>
       <c r="L51" s="22" t="n"/>
       <c r="M51" s="22" t="n"/>
@@ -3305,7 +3309,7 @@
         </is>
       </c>
       <c r="I52" s="155" t="n"/>
-      <c r="J52" s="128" t="n"/>
+      <c r="J52" s="157" t="n"/>
       <c r="K52" s="22" t="n"/>
       <c r="L52" s="22" t="n"/>
       <c r="M52" s="22" t="n"/>
@@ -3336,7 +3340,7 @@
         </is>
       </c>
       <c r="I53" s="155" t="n"/>
-      <c r="J53" s="128" t="n"/>
+      <c r="J53" s="157" t="n"/>
       <c r="K53" s="22" t="n"/>
       <c r="L53" s="22" t="n"/>
       <c r="M53" s="22" t="n"/>
@@ -3367,7 +3371,7 @@
         </is>
       </c>
       <c r="I54" s="155" t="n"/>
-      <c r="J54" s="128" t="n"/>
+      <c r="J54" s="157" t="n"/>
       <c r="K54" s="22" t="n"/>
       <c r="L54" s="22" t="n"/>
       <c r="M54" s="22" t="n"/>
@@ -3398,7 +3402,7 @@
         </is>
       </c>
       <c r="I55" s="155" t="n"/>
-      <c r="J55" s="128" t="n"/>
+      <c r="J55" s="157" t="n"/>
       <c r="K55" s="22" t="n"/>
       <c r="L55" s="22" t="n"/>
       <c r="M55" s="22" t="n"/>
@@ -3429,7 +3433,7 @@
         </is>
       </c>
       <c r="I56" s="155" t="n"/>
-      <c r="J56" s="128" t="n"/>
+      <c r="J56" s="157" t="n"/>
       <c r="K56" s="22" t="n"/>
       <c r="L56" s="22" t="n"/>
       <c r="M56" s="22" t="n"/>
@@ -3460,7 +3464,7 @@
         </is>
       </c>
       <c r="I57" s="155" t="n"/>
-      <c r="J57" s="128" t="n"/>
+      <c r="J57" s="157" t="n"/>
       <c r="K57" s="22" t="n"/>
       <c r="L57" s="22" t="n"/>
       <c r="M57" s="22" t="n"/>
@@ -3492,7 +3496,7 @@
         </is>
       </c>
       <c r="I58" s="155" t="n"/>
-      <c r="J58" s="128" t="n"/>
+      <c r="J58" s="157" t="n"/>
       <c r="K58" s="22" t="n"/>
       <c r="L58" s="22" t="n"/>
       <c r="M58" s="22" t="n"/>
@@ -3523,7 +3527,7 @@
         </is>
       </c>
       <c r="I59" s="155" t="n"/>
-      <c r="J59" s="128" t="n"/>
+      <c r="J59" s="157" t="n"/>
       <c r="K59" s="22" t="n"/>
       <c r="L59" s="22" t="n"/>
       <c r="M59" s="22" t="n"/>
@@ -3554,7 +3558,7 @@
         </is>
       </c>
       <c r="I60" s="155" t="n"/>
-      <c r="J60" s="128" t="n"/>
+      <c r="J60" s="157" t="n"/>
       <c r="K60" s="22" t="n"/>
       <c r="L60" s="22" t="n"/>
       <c r="M60" s="22" t="n"/>
@@ -3586,7 +3590,7 @@
         </is>
       </c>
       <c r="I61" s="155" t="n"/>
-      <c r="J61" s="128" t="n"/>
+      <c r="J61" s="157" t="n"/>
       <c r="K61" s="22" t="n"/>
       <c r="L61" s="22" t="n"/>
       <c r="M61" s="22" t="n"/>
@@ -3617,7 +3621,7 @@
         </is>
       </c>
       <c r="I62" s="142" t="n"/>
-      <c r="J62" s="128" t="n"/>
+      <c r="J62" s="157" t="n"/>
       <c r="K62" s="22" t="n"/>
       <c r="L62" s="22" t="n"/>
       <c r="M62" s="22" t="n"/>
@@ -3648,7 +3652,7 @@
         </is>
       </c>
       <c r="I63" s="155" t="n"/>
-      <c r="J63" s="128" t="n"/>
+      <c r="J63" s="157" t="n"/>
       <c r="K63" s="22" t="n"/>
       <c r="L63" s="22" t="n"/>
       <c r="M63" s="22" t="n"/>
@@ -3679,7 +3683,7 @@
         </is>
       </c>
       <c r="I64" s="155" t="n"/>
-      <c r="J64" s="128" t="n"/>
+      <c r="J64" s="157" t="n"/>
       <c r="K64" s="22" t="n"/>
       <c r="L64" s="22" t="n"/>
       <c r="M64" s="22" t="n"/>
@@ -3710,7 +3714,7 @@
         </is>
       </c>
       <c r="I65" s="155" t="n"/>
-      <c r="J65" s="128" t="n"/>
+      <c r="J65" s="157" t="n"/>
       <c r="K65" s="22" t="n"/>
       <c r="L65" s="22" t="n"/>
       <c r="M65" s="22" t="n"/>
@@ -3741,7 +3745,7 @@
         </is>
       </c>
       <c r="I66" s="155" t="n"/>
-      <c r="J66" s="128" t="n"/>
+      <c r="J66" s="157" t="n"/>
       <c r="K66" s="22" t="n"/>
       <c r="L66" s="22" t="n"/>
       <c r="M66" s="22" t="n"/>
@@ -3772,7 +3776,7 @@
         </is>
       </c>
       <c r="I67" s="155" t="n"/>
-      <c r="J67" s="128" t="n"/>
+      <c r="J67" s="157" t="n"/>
       <c r="K67" s="22" t="n"/>
       <c r="L67" s="22" t="n"/>
       <c r="M67" s="22" t="n"/>
@@ -3803,7 +3807,7 @@
         </is>
       </c>
       <c r="I68" s="155" t="n"/>
-      <c r="J68" s="128" t="n"/>
+      <c r="J68" s="157" t="n"/>
       <c r="K68" s="22" t="n"/>
       <c r="L68" s="22" t="n"/>
       <c r="M68" s="22" t="n"/>
@@ -3834,7 +3838,7 @@
         </is>
       </c>
       <c r="I69" s="155" t="n"/>
-      <c r="J69" s="128" t="n"/>
+      <c r="J69" s="157" t="n"/>
       <c r="K69" s="22" t="n"/>
       <c r="L69" s="22" t="n"/>
       <c r="M69" s="22" t="n"/>
@@ -3865,7 +3869,7 @@
         </is>
       </c>
       <c r="I70" s="155" t="n"/>
-      <c r="J70" s="128" t="n"/>
+      <c r="J70" s="157" t="n"/>
       <c r="K70" s="22" t="n"/>
       <c r="L70" s="22" t="n"/>
       <c r="M70" s="22" t="n"/>
@@ -3896,7 +3900,7 @@
         </is>
       </c>
       <c r="I71" s="155" t="n"/>
-      <c r="J71" s="128" t="n"/>
+      <c r="J71" s="157" t="n"/>
       <c r="K71" s="22" t="n"/>
       <c r="L71" s="22" t="n"/>
       <c r="M71" s="22" t="n"/>
@@ -3927,7 +3931,7 @@
         </is>
       </c>
       <c r="I72" s="155" t="n"/>
-      <c r="J72" s="128" t="n"/>
+      <c r="J72" s="157" t="n"/>
       <c r="K72" s="22" t="n"/>
       <c r="L72" s="22" t="n"/>
       <c r="M72" s="22" t="n"/>
@@ -3958,7 +3962,7 @@
         </is>
       </c>
       <c r="I73" s="155" t="n"/>
-      <c r="J73" s="128" t="n"/>
+      <c r="J73" s="157" t="n"/>
       <c r="K73" s="22" t="n"/>
       <c r="L73" s="22" t="n"/>
       <c r="M73" s="22" t="n"/>
@@ -4017,7 +4021,7 @@
         </is>
       </c>
       <c r="I75" s="155" t="n"/>
-      <c r="J75" s="128" t="n"/>
+      <c r="J75" s="157" t="n"/>
       <c r="K75" s="20">
         <f>(K74)/(K74+L74+M74)</f>
         <v/>
@@ -4058,7 +4062,7 @@
         </is>
       </c>
       <c r="I76" s="155" t="n"/>
-      <c r="J76" s="128" t="n"/>
+      <c r="J76" s="157" t="n"/>
       <c r="K76" s="22" t="n"/>
       <c r="L76" s="22" t="n"/>
       <c r="M76" s="22" t="n"/>
@@ -4089,7 +4093,7 @@
         </is>
       </c>
       <c r="I77" s="155" t="n"/>
-      <c r="J77" s="128" t="n"/>
+      <c r="J77" s="157" t="n"/>
       <c r="K77" s="22" t="n"/>
       <c r="L77" s="22" t="n"/>
       <c r="M77" s="22" t="n"/>
@@ -4122,7 +4126,7 @@
         </is>
       </c>
       <c r="I78" s="156" t="n"/>
-      <c r="J78" s="128" t="n"/>
+      <c r="J78" s="157" t="n"/>
       <c r="K78" s="22" t="n"/>
       <c r="L78" s="22" t="n"/>
       <c r="M78" s="22" t="n"/>
@@ -4153,7 +4157,7 @@
         </is>
       </c>
       <c r="I79" s="155" t="n"/>
-      <c r="J79" s="128" t="n"/>
+      <c r="J79" s="157" t="n"/>
       <c r="K79" s="22" t="n"/>
       <c r="L79" s="22" t="n"/>
       <c r="M79" s="22" t="n"/>
@@ -4184,7 +4188,7 @@
         </is>
       </c>
       <c r="I80" s="155" t="n"/>
-      <c r="J80" s="128" t="n"/>
+      <c r="J80" s="157" t="n"/>
       <c r="K80" s="22" t="n"/>
       <c r="L80" s="22" t="n"/>
       <c r="M80" s="22" t="n"/>
@@ -4215,7 +4219,7 @@
         </is>
       </c>
       <c r="I81" s="155" t="n"/>
-      <c r="J81" s="128" t="n"/>
+      <c r="J81" s="157" t="n"/>
       <c r="K81" s="22" t="n"/>
       <c r="L81" s="22" t="n"/>
       <c r="M81" s="22" t="n"/>
@@ -4246,7 +4250,7 @@
         </is>
       </c>
       <c r="I82" s="155" t="n"/>
-      <c r="J82" s="128" t="n"/>
+      <c r="J82" s="157" t="n"/>
       <c r="K82" s="22" t="n"/>
       <c r="L82" s="22" t="n"/>
       <c r="M82" s="22" t="n"/>
@@ -4277,7 +4281,7 @@
         </is>
       </c>
       <c r="I83" s="155" t="n"/>
-      <c r="J83" s="128" t="n"/>
+      <c r="J83" s="157" t="n"/>
       <c r="K83" s="22" t="n"/>
       <c r="L83" s="22" t="n"/>
       <c r="M83" s="22" t="n"/>
@@ -4309,7 +4313,7 @@
         </is>
       </c>
       <c r="I84" s="155" t="n"/>
-      <c r="J84" s="128" t="n"/>
+      <c r="J84" s="157" t="n"/>
       <c r="K84" s="22" t="n"/>
       <c r="L84" s="22" t="n"/>
       <c r="M84" s="22" t="n"/>
@@ -4340,7 +4344,7 @@
         </is>
       </c>
       <c r="I85" s="155" t="n"/>
-      <c r="J85" s="128" t="n"/>
+      <c r="J85" s="157" t="n"/>
       <c r="K85" s="22" t="n"/>
       <c r="L85" s="22" t="n"/>
       <c r="M85" s="22" t="n"/>
@@ -4371,7 +4375,7 @@
         </is>
       </c>
       <c r="I86" s="155" t="n"/>
-      <c r="J86" s="128" t="n"/>
+      <c r="J86" s="157" t="n"/>
       <c r="K86" s="22" t="n"/>
       <c r="L86" s="22" t="n"/>
       <c r="M86" s="22" t="n"/>
@@ -4407,7 +4411,7 @@
           <t>Abertura de Plano de Ação para desvios de metas em Junho.</t>
         </is>
       </c>
-      <c r="J87" s="128" t="n"/>
+      <c r="J87" s="157" t="n"/>
       <c r="K87" s="22" t="n"/>
       <c r="L87" s="22" t="n"/>
       <c r="M87" s="22" t="n"/>
@@ -4438,7 +4442,7 @@
         </is>
       </c>
       <c r="I88" s="155" t="n"/>
-      <c r="J88" s="128" t="n"/>
+      <c r="J88" s="157" t="n"/>
       <c r="K88" s="22" t="n"/>
       <c r="L88" s="22" t="n"/>
       <c r="M88" s="22" t="n"/>
@@ -4469,7 +4473,7 @@
         </is>
       </c>
       <c r="I89" s="155" t="n"/>
-      <c r="J89" s="128" t="n"/>
+      <c r="J89" s="157" t="n"/>
       <c r="K89" s="22" t="n"/>
       <c r="L89" s="22" t="n"/>
       <c r="M89" s="22" t="n"/>
@@ -9559,7 +9563,7 @@
       <c r="AE43" s="66" t="n"/>
       <c r="AF43" s="66" t="n"/>
     </row>
-    <row r="44" ht="17.25" customHeight="1" s="104">
+    <row r="44" ht="20" customHeight="1" s="104">
       <c r="A44" s="66" t="n"/>
       <c r="B44" s="55" t="inlineStr">
         <is>
@@ -9574,7 +9578,7 @@
         <f>H4</f>
         <v/>
       </c>
-      <c r="E44" s="146" t="n"/>
+      <c r="E44" s="158" t="inlineStr"/>
       <c r="F44" s="127" t="n"/>
       <c r="G44" s="127" t="n"/>
       <c r="H44" s="127" t="n"/>
@@ -9603,7 +9607,7 @@
       <c r="AE44" s="66" t="n"/>
       <c r="AF44" s="66" t="n"/>
     </row>
-    <row r="45" ht="12.75" customHeight="1" s="104">
+    <row r="45" ht="20" customHeight="1" s="104">
       <c r="A45" s="66" t="n"/>
       <c r="B45" s="55" t="inlineStr">
         <is>
@@ -9618,7 +9622,7 @@
         <f>H5</f>
         <v/>
       </c>
-      <c r="E45" s="147" t="n"/>
+      <c r="E45" s="158" t="inlineStr"/>
       <c r="F45" s="127" t="n"/>
       <c r="G45" s="127" t="n"/>
       <c r="H45" s="127" t="n"/>
@@ -9647,7 +9651,7 @@
       <c r="AE45" s="66" t="n"/>
       <c r="AF45" s="66" t="n"/>
     </row>
-    <row r="46" ht="12.75" customHeight="1" s="104">
+    <row r="46" ht="20" customHeight="1" s="104">
       <c r="A46" s="66" t="n"/>
       <c r="B46" s="55" t="inlineStr">
         <is>
@@ -9662,7 +9666,7 @@
         <f>H6</f>
         <v/>
       </c>
-      <c r="E46" s="147" t="n"/>
+      <c r="E46" s="158" t="inlineStr"/>
       <c r="F46" s="127" t="n"/>
       <c r="G46" s="127" t="n"/>
       <c r="H46" s="127" t="n"/>
@@ -9691,7 +9695,7 @@
       <c r="AE46" s="66" t="n"/>
       <c r="AF46" s="66" t="n"/>
     </row>
-    <row r="47" ht="12.75" customHeight="1" s="104">
+    <row r="47" ht="20" customHeight="1" s="104">
       <c r="A47" s="66" t="n"/>
       <c r="B47" s="55" t="inlineStr">
         <is>
@@ -9706,7 +9710,7 @@
         <f>H7</f>
         <v/>
       </c>
-      <c r="E47" s="147" t="n"/>
+      <c r="E47" s="158" t="inlineStr"/>
       <c r="F47" s="127" t="n"/>
       <c r="G47" s="127" t="n"/>
       <c r="H47" s="127" t="n"/>
@@ -9735,7 +9739,7 @@
       <c r="AE47" s="66" t="n"/>
       <c r="AF47" s="66" t="n"/>
     </row>
-    <row r="48" ht="12.75" customHeight="1" s="104">
+    <row r="48" ht="36" customHeight="1" s="104">
       <c r="A48" s="66" t="n"/>
       <c r="B48" s="55" t="inlineStr">
         <is>
@@ -9750,7 +9754,11 @@
         <f>H8</f>
         <v/>
       </c>
-      <c r="E48" s="147" t="n"/>
+      <c r="E48" s="158" t="inlineStr">
+        <is>
+          <t>• Item 8.5.1 [NC]: KPI - SERVICE RATE: Meta &gt;=95% | Realizado: Junho: 91,17% / KPI - LATE ORDERS: Meta &lt;=2,00% | Realizado: Junho: 4,32%</t>
+        </is>
+      </c>
       <c r="F48" s="127" t="n"/>
       <c r="G48" s="127" t="n"/>
       <c r="H48" s="127" t="n"/>

</xml_diff>